<commit_message>
fix: use yes-no values in database templates
</commit_message>
<xml_diff>
--- a/docs/database/import-templates/DB-01-user-profiles.xlsx
+++ b/docs/database/import-templates/DB-01-user-profiles.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R4a7d9cf4431d43b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rbe7e2407a0d74419"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -660,7 +660,7 @@
       <x:alignment vertical="center"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="18">
+  <x:cellXfs count="15">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -682,14 +682,6 @@
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <x:alignment vertical="center"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
-      <x:alignment vertical="center"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
-    </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -701,14 +693,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
@@ -721,14 +705,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-      <x:extLst>
-        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
-        </x:ext>
-      </x:extLst>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="49">
@@ -783,23 +759,6 @@
     <x:cellStyle name="60% - 强调文字颜色 6" xfId="48"/>
   </x:cellStyles>
 </x:styleSheet>
-</file>
-
-<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
-<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
-  <xfpb:bag type="Checkbox"/>
-  <xfpb:bag type="XFControls">
-    <xfpb:bagId k="CellControl">0</xfpb:bagId>
-  </xfpb:bag>
-  <xfpb:bag type="XFComplement">
-    <xfpb:bagId k="XFControls">1</xfpb:bagId>
-  </xfpb:bag>
-  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
-    <xfpb:a k="MappedFeaturePropertyBags">
-      <xfpb:bagId>2</xfpb:bagId>
-    </xfpb:a>
-  </xfpb:bag>
-</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1028,118 +987,118 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
-      <x:c r="A1" s="13" t="s">
+      <x:c r="A1" s="11" t="s">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="B1" s="14" t="s">
+      <x:c r="B1" s="12" t="s">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C1" s="14" t="s">
+      <x:c r="C1" s="12" t="s">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D1" s="14" t="s">
+      <x:c r="D1" s="12" t="s">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="E1" s="15" t="s">
+      <x:c r="E1" s="13" t="s">
         <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="30" customHeight="1">
-      <x:c r="A2" s="16" t="str">
+      <x:c r="A2" s="14" t="str">
         <x:v>profile_json</x:v>
       </x:c>
-      <x:c r="B2" s="16" t="str">
+      <x:c r="B2" s="14" t="str">
         <x:v>String</x:v>
       </x:c>
-      <x:c r="C2" s="16" t="str">
+      <x:c r="C2" s="14" t="str">
         <x:v>已由用户确认的正式画像 JSON</x:v>
       </x:c>
-      <x:c r="D2" s="16" t="str">
+      <x:c r="D2" s="14" t="str">
         <x:v>{}</x:v>
       </x:c>
-      <x:c r="E2" s="17" t="b">
-        <x:v>0</x:v>
+      <x:c r="E2" s="14" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
-      <x:c r="A3" s="16" t="str">
+      <x:c r="A3" s="14" t="str">
         <x:v>pending_profile_json</x:v>
       </x:c>
-      <x:c r="B3" s="16" t="str">
+      <x:c r="B3" s="14" t="str">
         <x:v>String</x:v>
       </x:c>
-      <x:c r="C3" s="16" t="str">
+      <x:c r="C3" s="14" t="str">
         <x:v>等待用户确认的画像草稿 JSON</x:v>
       </x:c>
-      <x:c r="D3" s="16" t="str">
+      <x:c r="D3" s="14" t="str">
         <x:v>{}</x:v>
       </x:c>
-      <x:c r="E3" s="17" t="b">
-        <x:v>0</x:v>
+      <x:c r="E3" s="14" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="30" customHeight="1">
-      <x:c r="A4" s="16" t="str">
+      <x:c r="A4" s="14" t="str">
         <x:v>confirmation_token</x:v>
       </x:c>
-      <x:c r="B4" s="16" t="str">
+      <x:c r="B4" s="14" t="str">
         <x:v>String</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="str">
+      <x:c r="C4" s="14" t="str">
         <x:v>当前待确认草稿的令牌</x:v>
       </x:c>
-      <x:c r="D4" s="16"/>
-      <x:c r="E4" s="17" t="b">
-        <x:v>0</x:v>
+      <x:c r="D4" s="14"/>
+      <x:c r="E4" s="14" t="str">
+        <x:v>否</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
-      <x:c r="A5" s="16" t="str">
+      <x:c r="A5" s="14" t="str">
         <x:v>pending_status</x:v>
       </x:c>
-      <x:c r="B5" s="16" t="str">
+      <x:c r="B5" s="14" t="str">
         <x:v>String</x:v>
       </x:c>
-      <x:c r="C5" s="16" t="str">
+      <x:c r="C5" s="14" t="str">
         <x:v>none/awaiting_confirmation/confirmed/expired</x:v>
       </x:c>
-      <x:c r="D5" s="16" t="str">
+      <x:c r="D5" s="14" t="str">
         <x:v>none</x:v>
       </x:c>
-      <x:c r="E5" s="17" t="b">
-        <x:v>1</x:v>
+      <x:c r="E5" s="14" t="str">
+        <x:v>是</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="30" customHeight="1">
-      <x:c r="A6" s="16" t="str">
+      <x:c r="A6" s="14" t="str">
         <x:v>record_version</x:v>
       </x:c>
-      <x:c r="B6" s="16" t="str">
+      <x:c r="B6" s="14" t="str">
         <x:v>Integer</x:v>
       </x:c>
-      <x:c r="C6" s="16" t="str">
+      <x:c r="C6" s="14" t="str">
         <x:v>画像记录版本号</x:v>
       </x:c>
-      <x:c r="D6" s="16" t="n">
+      <x:c r="D6" s="14" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E6" s="17" t="b">
-        <x:v>1</x:v>
+      <x:c r="E6" s="14" t="str">
+        <x:v>是</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="30" customHeight="1">
-      <x:c r="A7" s="16" t="str">
+      <x:c r="A7" s="14" t="str">
         <x:v>updated_at</x:v>
       </x:c>
-      <x:c r="B7" s="16" t="str">
+      <x:c r="B7" s="14" t="str">
         <x:v>Time</x:v>
       </x:c>
-      <x:c r="C7" s="16" t="str">
+      <x:c r="C7" s="14" t="str">
         <x:v>最后修改时间</x:v>
       </x:c>
-      <x:c r="D7" s="16"/>
-      <x:c r="E7" s="17" t="b">
-        <x:v>1</x:v>
+      <x:c r="D7" s="14"/>
+      <x:c r="E7" s="14" t="str">
+        <x:v>是</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: migrate databases to internal user keys
</commit_message>
<xml_diff>
--- a/docs/database/import-templates/DB-01-user-profiles.xlsx
+++ b/docs/database/import-templates/DB-01-user-profiles.xlsx
@@ -1205,7 +1205,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>profile_json</t>
+          <t>user_key</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1215,24 +1215,20 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>已由用户确认的正式画像 JSON</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
+          <t>MAIN 生成的会话级业务用户键</t>
+        </is>
+      </c>
+      <c r="D2"/>
       <c r="E2" t="inlineStr">
         <is>
-          <t>否</t>
+          <t>是</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>pending_profile_json</t>
+          <t>profile_json</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1242,7 +1238,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>等待用户确认的画像草稿 JSON</t>
+          <t>已由用户确认的正式画像 JSON</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1259,7 +1255,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>confirmation_token</t>
+          <t>pending_profile_json</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1269,10 +1265,14 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>当前待确认草稿的令牌</t>
-        </is>
-      </c>
-      <c r="D4"/>
+          <t>等待用户确认的画像草稿 JSON</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>否</t>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>none/awaiting_confirmation/confirmed/expired</t>
+          <t>none/awaiting_confirmation/confirmed/cancelled</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1336,20 +1336,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>source_workflow</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Time</t>
+          <t>String</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>最后修改时间</t>
-        </is>
-      </c>
-      <c r="D7"/>
+          <t>固定 WF-01</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>WF-01</t>
+        </is>
+      </c>
       <c r="E7" t="inlineStr">
         <is>
           <t>是</t>

</xml_diff>